<commit_message>
Rerun with contamination-aware panels; Figure 5 legend tidy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/results/pathways/BC_vs_Control/mcg_modularanalysis_BC_vs_Control.xlsx
+++ b/results/pathways/BC_vs_Control/mcg_modularanalysis_BC_vs_Control.xlsx
@@ -37,10 +37,10 @@
     <t>module_1</t>
   </si>
   <si>
-    <t>3beta-Hydroxyandrost-5-en-17-one; Dehydroepiandrosterone; Dehydroisoandrosterone; DHA; DHEA$Cortisol; Hydrocortisone; 11beta,17alpha,21-Trihydroxy-4-pregnene-3,20-dione; Kendall's compound F; Reichstein's substance M$16alpha-Hydroxydehydroepiandrosterone; 5-Androstene-3beta,16alpha-diol-17-one$11-Deoxycorticosterone; Deoxycorticosterone; Cortexone; 21-Hydroxy-4-pregnene-3,20-dione; Desoxycortone; DOC$11-Deoxycortisol; Cortodoxone$Androst-5-ene-3beta,17beta-diol; 3beta,17beta-Dihydroxyandrost-5-ene; 3beta,17beta-Dihydroxy-5-androstene; Androstenediol$17alpha-Hydroxyprogesterone; 17alpha-Hydroxy-4-pregnene-3,20-dione; Pregn-4-ene-3,20-dione-17-ol; 17alpha-Hydroxy-progesterone$11beta-Hydroxyprogesterone$11beta,17alpha,21-Trihydroxypregnenolone$17alpha,21-Dihydroxypregnenolone$$Pregnenolone; 5-Pregnen-3beta-ol-20-one; 3beta-Hydroxypregn-5-en-20-one$18-Hydroxycorticosterone$21-Deoxycortisol; 4-Pregnene-11beta,17alpha-diol-3,20-dione; 11beta,17alpha-Dihydroxyprogesterone</t>
-  </si>
-  <si>
-    <t>C01227,C00735,C05139,C03205,C05488,C04295,C01176,C05498,C05489,C05487,C18045,C01953,C01124,C05497</t>
+    <t>Cortisol; Hydrocortisone; 11beta,17alpha,21-Trihydroxy-4-pregnene-3,20-dione; Kendall's compound F; Reichstein's substance M$11-Deoxycortisol; Cortodoxone$16alpha-Hydroxydehydroepiandrosterone; 5-Androstene-3beta,16alpha-diol-17-one$17alpha-Hydroxyprogesterone; 17alpha-Hydroxy-4-pregnene-3,20-dione; Pregn-4-ene-3,20-dione-17-ol; 17alpha-Hydroxy-progesterone$11beta,17alpha,21-Trihydroxypregnenolone$11beta-Hydroxyprogesterone$3beta-Hydroxyandrost-5-en-17-one; Dehydroepiandrosterone; Dehydroisoandrosterone; DHA; DHEA$21-Deoxycortisol; 4-Pregnene-11beta,17alpha-diol-3,20-dione; 11beta,17alpha-Dihydroxyprogesterone$18-Hydroxycorticosterone$Androst-5-ene-3beta,17beta-diol; 3beta,17beta-Dihydroxyandrost-5-ene; 3beta,17beta-Dihydroxy-5-androstene; Androstenediol$$Pregnenolone; 5-Pregnen-3beta-ol-20-one; 3beta-Hydroxypregn-5-en-20-one$11-Deoxycorticosterone; Deoxycorticosterone; Cortexone; 21-Hydroxy-4-pregnene-3,20-dione; Desoxycortone; DOC$17alpha,21-Dihydroxypregnenolone</t>
+  </si>
+  <si>
+    <t>C00735,C05488,C05139,C01176,C05489,C05498,C01227,C05497,C01124,C04295,C18045,C01953,C03205,C05487</t>
   </si>
   <si>
     <t>(12, 'C21-steroid hormone biosynthesis and metabolism');(5, 'Androgen and estrogen biosynthesis and metabolism')</t>
@@ -403,7 +403,7 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>0.04914085586078581</v>
+        <v>0.0471956975085062</v>
       </c>
       <c r="C2">
         <v>14</v>

</xml_diff>

<commit_message>
Full re-run with stage-2 ages; MSI levels from MS2 library matches; updated figures, tables, draft text
- 41/45 controls with age: 18 BC-Control pairs, 295 adjusted-significant compounds, 212 findings
- Val-Leu (stage-1 marker) replicated (q = 0.048, age-matched p = 0.004)
- MSI 2/3/4 rule uses MS-DIAL MS2 library flags (curation/ms2_identified.csv)
- Figure 4 limited to 50 findings; README and manuscript draft numbers updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/results/pathways/BC_vs_Control/mcg_modularanalysis_BC_vs_Control.xlsx
+++ b/results/pathways/BC_vs_Control/mcg_modularanalysis_BC_vs_Control.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>MODULE</t>
   </si>
@@ -32,18 +32,6 @@
   </si>
   <si>
     <t>This module overlaps with</t>
-  </si>
-  <si>
-    <t>module_1</t>
-  </si>
-  <si>
-    <t>Cortisol; Hydrocortisone; 11beta,17alpha,21-Trihydroxy-4-pregnene-3,20-dione; Kendall's compound F; Reichstein's substance M$11-Deoxycortisol; Cortodoxone$16alpha-Hydroxydehydroepiandrosterone; 5-Androstene-3beta,16alpha-diol-17-one$17alpha-Hydroxyprogesterone; 17alpha-Hydroxy-4-pregnene-3,20-dione; Pregn-4-ene-3,20-dione-17-ol; 17alpha-Hydroxy-progesterone$11beta,17alpha,21-Trihydroxypregnenolone$11beta-Hydroxyprogesterone$3beta-Hydroxyandrost-5-en-17-one; Dehydroepiandrosterone; Dehydroisoandrosterone; DHA; DHEA$21-Deoxycortisol; 4-Pregnene-11beta,17alpha-diol-3,20-dione; 11beta,17alpha-Dihydroxyprogesterone$18-Hydroxycorticosterone$Androst-5-ene-3beta,17beta-diol; 3beta,17beta-Dihydroxyandrost-5-ene; 3beta,17beta-Dihydroxy-5-androstene; Androstenediol$$Pregnenolone; 5-Pregnen-3beta-ol-20-one; 3beta-Hydroxypregn-5-en-20-one$11-Deoxycorticosterone; Deoxycorticosterone; Cortexone; 21-Hydroxy-4-pregnene-3,20-dione; Desoxycortone; DOC$17alpha,21-Dihydroxypregnenolone</t>
-  </si>
-  <si>
-    <t>C00735,C05488,C05139,C01176,C05489,C05498,C01227,C05497,C01124,C04295,C18045,C01953,C03205,C05487</t>
-  </si>
-  <si>
-    <t>(12, 'C21-steroid hormone biosynthesis and metabolism');(5, 'Androgen and estrogen biosynthesis and metabolism')</t>
   </si>
 </sst>
 </file>
@@ -375,7 +363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -398,26 +386,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>0.0471956975085062</v>
-      </c>
-      <c r="C2">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>